<commit_message>
feat: add Excel import functionality for travel requests with template generation and parsing utilities
</commit_message>
<xml_diff>
--- a/public/modelo-solicitacao-viagem.xlsx
+++ b/public/modelo-solicitacao-viagem.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:M2"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -412,8 +412,6 @@
     <col min="11" max="11" width="22.83203125" customWidth="1"/>
     <col min="12" max="12" width="22.83203125" customWidth="1"/>
     <col min="13" max="13" width="22.83203125" customWidth="1"/>
-    <col min="14" max="14" width="22.83203125" customWidth="1"/>
-    <col min="15" max="15" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -436,30 +434,24 @@
         <v>E-mail Institucional</v>
       </c>
       <c r="G1" t="str">
-        <v>Justificativa do Interesse Público</v>
+        <v>Destino</v>
       </c>
       <c r="H1" t="str">
-        <v>Nexo com as Atribuições do Cargo</v>
+        <v>Data de Ida</v>
       </c>
       <c r="I1" t="str">
-        <v>Destino</v>
+        <v>Data de Volta</v>
       </c>
       <c r="J1" t="str">
-        <v>Data de Ida</v>
+        <v>Justificativa de Localização</v>
       </c>
       <c r="K1" t="str">
-        <v>Data de Volta</v>
+        <v>Indicação de Voo</v>
       </c>
       <c r="L1" t="str">
-        <v>Justificativa de Localização</v>
+        <v>Indicação de Hospedagem</v>
       </c>
       <c r="M1" t="str">
-        <v>Indicação de Voo</v>
-      </c>
-      <c r="N1" t="str">
-        <v>Indicação de Hospedagem</v>
-      </c>
-      <c r="O1" t="str">
         <v>Ficha Orçamentária</v>
       </c>
     </row>
@@ -483,36 +475,30 @@
         <v>joao.silva@osasco.sp.gov.br</v>
       </c>
       <c r="G2" t="str">
-        <v>Participação em congresso nacional de gestão pública para capacitação da equipe.</v>
+        <v>Brasília, DF</v>
       </c>
       <c r="H2" t="str">
-        <v>O cargo de Analista de Políticas Públicas exige atualização constante em gestão municipal.</v>
+        <v>20/04/2026</v>
       </c>
       <c r="I2" t="str">
-        <v>Brasília, DF</v>
+        <v>23/04/2026</v>
       </c>
       <c r="J2" t="str">
-        <v>20/04/2026</v>
+        <v>O evento ocorre exclusivamente em Brasília, sede do governo federal.</v>
       </c>
       <c r="K2" t="str">
-        <v>23/04/2026</v>
+        <v>Voo das 06h30 (LATAM LA3456)</v>
       </c>
       <c r="L2" t="str">
-        <v>O evento ocorre exclusivamente em Brasília, sede do governo federal.</v>
+        <v>Hotel próximo ao centro de convenções</v>
       </c>
       <c r="M2" t="str">
-        <v>Voo das 06h30 (LATAM LA3456)</v>
-      </c>
-      <c r="N2" t="str">
-        <v>Hotel próximo ao centro de convenções</v>
-      </c>
-      <c r="O2" t="str">
         <v>02.10.01.001</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>